<commit_message>
Refine contract generator: cleaner fields, auto-derive plot caps, add README
https://claude.ai/code/session_01XNwruHkNzzkACBuMPFnptn
</commit_message>
<xml_diff>
--- a/customers_template.xlsx
+++ b/customers_template.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -531,6 +531,11 @@
           <t>PAYMENT_START_DAY_FULL</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>NUM_PLOTS_WORDS_UPPER</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>

<commit_message>
Sync customers template and generator script updates
https://claude.ai/code/session_01XNwruHkNzzkACBuMPFnptn
</commit_message>
<xml_diff>
--- a/customers_template.xlsx
+++ b/customers_template.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,123 +413,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="41" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="37" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="48" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="27" customWidth="1" min="16" max="16"/>
-    <col width="27" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>CONTRACT_DAY</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CONTRACT_MONTH</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>CONTRACT_YEAR</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>CUSTOMER_NAME</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>CUSTOMER_ADDRESS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NUM_PLOTS_WORDS</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>NUM_PLOTS_DIGITS</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>PLOT_SIZE_SQM</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TOTAL_PRICE_DIGITS</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>TOTAL_PRICE_WORDS</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>DEPOSIT_DIGITS</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>DEPOSIT_WORDS</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>BALANCE_DIGITS</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>BALANCE_WORDS</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>PAYMENT_START_DATE</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>PAYMENT_DURATION_MONTHS</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>PAYMENT_END_DATE</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>PAYMENT_START_DAY_FULL</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>NUM_PLOTS_WORDS_UPPER</t>
         </is>
       </c>
     </row>
@@ -560,7 +531,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>9, OYEBANKE OSUNSANYA CRESCENT, LAGOS</t>
+          <t>9 OYEBANKE OSUNSANYA CRESCENT LAGOS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -580,7 +551,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>3000000</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -590,7 +561,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>800,000.00</t>
+          <t>800000.00</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -600,17 +571,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2,200,000.00</t>
+          <t>2200000.00</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>TWO MILLION, TWO HUNDRED THOUSAND NAIRA ONLY</t>
+          <t>TWO MILLION TWO HUNDRED THOUSAND NAIRA ONLY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>26th March, 2026</t>
+          <t>26th March 2026</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -620,12 +591,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>26th Day of March, 2027</t>
+          <t>26th Day of March 2027</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>26TH MARCH, 2027</t>
+          <t>26TH MARCH 2027</t>
         </is>
       </c>
     </row>

</xml_diff>